<commit_message>
ran initial panel regression model. pending validation tests
</commit_message>
<xml_diff>
--- a/data/interim/exposure_coding.xlsx
+++ b/data/interim/exposure_coding.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="34400" windowHeight="28200" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="coding" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="source_register" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="source_to_waves" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="coding" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="source_register" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="source_to_waves" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
finished robustness checks and data validation
</commit_message>
<xml_diff>
--- a/data/interim/exposure_coding.xlsx
+++ b/data/interim/exposure_coding.xlsx
@@ -10,15 +10,18 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="source_register" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="source_to_waves" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <definedNames>
+    <definedName name="source_register" localSheetId="1">source_register!$A$1:$K$32</definedName>
+  </definedNames>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -51,95 +54,16 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="23">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="yyyy/mm/dd"/>
-      <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="yyyy/mm/dd"/>
-      <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -210,25 +134,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table3" displayName="Table3" ref="A1:I1048576" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:I1048576"/>
-  <tableColumns count="10">
-    <tableColumn id="1" name="source_id"/>
-    <tableColumn id="2" name="full_citation"/>
-    <tableColumn id="3" name="type"/>
-    <tableColumn id="4" name="published"/>
-    <tableColumn id="5" name="activity_start"/>
-    <tableColumn id="10" name="activity_end"/>
-    <tableColumn id="11" name="countries"/>
-    <tableColumn id="6" name="independence"/>
-    <tableColumn id="7" name="local_path"/>
-    <tableColumn id="8" name="Column2"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -12098,64 +12003,1662 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="15.83203125" customWidth="1" style="3" min="1" max="9"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="80.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="41.6640625" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="19.5" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="11.1640625" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="10.5" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="80.6640625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="11.83203125" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="19.6640625" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="80.6640625" bestFit="1" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>source_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>full_citation</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>published</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>activity_start</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>activity_end</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>countries</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>independence</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>local_path</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>online_url</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>EDL22</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Doppelganger: Media clones serving Russian Propaganda</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>EU DisinfoLab</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>NGO / Research</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>44831</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>44682</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>44805</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC; IT ABC; FR ABC; LV ABC; LT AB; EE AB</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>sources/EDL22.pdf</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.disinfo.eu/doppelganger</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>DFR22</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Russia-based Facebook operation targeted Europe with anti-Ukraine messaging</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>DFRLab</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>NGO / Research</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>44831</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>44621</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>44774</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC; FR ABC; IT ABC; LV ABC; PL AC</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>sources/DFR22.pdf</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>https://dfrlab.org/2022/09/27/russia-based-facebook-operation-targeted-europe-with-anti-ukraine-messaging/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>MET22</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Removing Coordinated Inauthentic Behavior From China and Russia</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Platform Disclosure</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>44831</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>44682</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>44896</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC; FR ABC; IT ABC; LV AB</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>sources/MET22.pdf</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>https://about.fb.com/news/2022/09/removing-coordinated-inauthentic-behavior-from-china-and-russia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>ISD22</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Pro-Kremlin network impersonates legitimate websites and floods social media with lies</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Institute for Strategic Dialogue</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>NGO / Research</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>44833</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>44713</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>44796</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC; FR ABC; IT ABC</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>sources/ISD22.pdf</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.isdglobal.org/digital-dispatch/pro-kremlin-network-impersonates-legitimate-websites-and-floods-social-media-with-lies/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>VIG23</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>RRN: A complex and persistent information manipulation campaign ‚Äì¬†technical report</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>VIGINUM</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>State Forensic</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>45126</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>44958</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>45078</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>FR ABC; DE ABC</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>sources/VIG23.pdf</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sgdsn.gouv.fr/publications/maj-19062023-rrn-une-campagne-numerique-de-manipulation-de-linformation-complexe-et</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>RST23</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Under the Radar: Vast Networks of Fake Accounts Raise Questions About Meta‚Äôs Compliance with the EU‚Äôs New Digital Rulebook.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Reset Tech</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>NGO / Research</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>45139</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>44927</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>45017</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC; FR ABC; IT C</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>sources/RST23.pdf</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reset.tech/resources/vast-networks-of-fake-accounts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>MET23</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Adversarial Threat Report, Second Quarter</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Platform Disclosure</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>45139</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>45017</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>45078</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC; FR ABC; PL ABC</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>sources/MET23.pdf</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>https://transparency.meta.com/sr/Q2-2023-Adversarial-threat-report/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>VIG24</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Portal Kombat: A structured and coordinated pro-Russian propaganda network</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>VIGINUM</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>State Forensic</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>45334</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>45170</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>45261</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC; FR ABC; AT ABC; PL ABC; ES ABC</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>sources/VIG24.pdf</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sgdsn.gouv.fr/files/files/20240212_NP_SGDSN_VIGINUM_PORTAL-KOMBAT-NETWORK_ENG_VF.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>AIF24</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>No Embargo in Sight: Meta lets Pro-Russia Propaganda Ads Flood the EU</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>AI Forensics</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>NGO / Research</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>45399</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>45155</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>45382</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>DE AC; FR AC</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>sources/AIF24.pdf</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>https://aiforensics.org/work/meta-political-ads</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>AIF24-2</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Supporting Evidence: Pro-Russian Ads Campaigns Approved by Meta from May 1 to May 27, 2024 in Italy, Germany, France &amp; Poland</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>AI Forensics</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>NGO / Research</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>45439</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>45413</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>45439</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>DE: AC; FR AC; IT AC; PL AC</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>sources/AIF24-2.pdf</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>https://cmsbackend.aiforensics.org/uploads/Meta_Ads_Follow_up_27_May_24_46d87a3953.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>SEK24</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Master of Puppets: Uncovering the DoppelG√§nger pro-Russian influence campaign</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Sekoia</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Commercial Threat Intel</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>45433</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>45231</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>45383</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>FR ABC; DE ABC; LT A; IT AC; SK A</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>sources/SEK24.pdf</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sekoia.com/blog/master-of-puppets-uncovering-the-doppelganger-pro-russian-influence-campaign#toc-3-i-doppelgnger-campaign-victims-objective</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>MET24</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Adversarial Threat Report, Second Quarter</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Platform Disclosure</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>45505</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>45383</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>45444</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>DE AC; FR AC; PL AC</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>sources/MET24.pdf</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>https://transparency.meta.com/sr/Q2-2024-Adversarial-threat-report/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>OAI24</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>AI and Covert Influence Operations: Latest Trends</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Platform Disclosure</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>45442</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>45323</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>45383</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>DE AC; FR AC; PL AC; IT AC</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>sources/OAI24.pdf</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>https://openai.com/index/disrupting-deceptive-uses-of-ai-by-covert-influence-operations/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>EDM24</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Russian disinformation network ‚ÄúPravda‚Äù grew bigger in the EU, even after its uncovering</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>European Digital Media Observatory</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>NGO / Research</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>45406</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>45352</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>45383</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>EL AC; IT AC; NL AC; DK AC; HR AC; CZ AC; SK AC; BG AC; RO AC; FI AC; SE AC; PT AC; EE AC; LV AC; LT AC; HU AC; CY AC; IE AC; SI AC</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>sources/EDM24.pdf</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>https://edmo.eu/publications/russian-disinformation-network-pravda-grew-bigger-in-the-eu-even-after-its-uncovering/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>CHK24</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Operation Overload: how pro-Russian actors flood newsrooms with fake content and seek to divert their efforts</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>CheckFirst</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Commercial Threat Intel</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>45447</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>45139</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>45383</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC; FR ABC</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>sources/CHK24.pdf</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>https://checkfirst.network/operation-overload-how-pro-russian-actors-flood-newsrooms-with-fake-content-and-seek-to-divert-their-efforts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>VIG24-2</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Matryoshka: A pro-Russian campaign targeting media and the fact-checking community</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>VIGINUM</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>State Forensic</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>45454</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>45174</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>45444</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>FR ABC; DE AC; IT AC</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>sources/VIG24-2.pdf</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sgdsn.gouv.fr/files/files/20240611_NP_SGDSN_VIGINUM_Matriochka_EN_VF.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>FFO24</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Germany Targeted by the Pro-Russian Disinformation Campaign ‚ÄúDoppelg√§nger‚Äù</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>German Federal Foreign Office</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>State Forensic</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>45448</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>44986</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>45437</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>sources/FFO24.pdf</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.auswaertiges-amt.de/resource/blob/2682484/2da31936d1cbeb9faec49df74d8bbe2e/technischer-bericht-desinformationskampagne-doppelgaenger-1--data.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>EAS24</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Doppelganger strikes back: FIMI activities in the context of the EE24</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>European External Action Service</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>State Forensic</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>45462</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>44980</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>45444</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC; FR ABC; IT ABC; PL ABC; ES ABC</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>sources/EAS24.pdf</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>https://euvsdisinfo.eu/uploads/2024/06/EEAS-TechnicalReport-DoppelgangerEE24_June2024.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>DFR24</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Doppelganger targets Ukrainian and French audiences via Facebook ads</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>DFRLab</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>NGO / Research</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>45363</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>45108</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>45323</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>FR ABC; DE ABC</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>sources/DFR24.pdf</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>https://dfrlab.org/2024/03/12/doppelganger-operation-targets-ukraine/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>HFL24</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Mid-year Doppelganger Information Operations in Europe and the US</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>HarfangLab</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Commercial Threat Intel</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>45498</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>45413</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>45474</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>FR ABC; DE ABC; PL AC; HU A</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>sources/HFL24.pdf</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>https://harfanglab.io/insidethelab/doppelganger-operations-europe-us/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>BLV24-ENG</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Internal Details on the Russian Disinformation Campaign "Doppelg√§nger"</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Bavarian Office for the Protection of the Constitution</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>State Forensic</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>45505</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>45047</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>45474</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC; FR ABC; PL AC; IT AC; ES AC</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>sources/BLV24-ENG.pdf</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lfv.bayern.de/wp-content/uploads/2025/05/baylfv_vollanalyse_doppelgaenger.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>SNT24</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Doppelg√§nger | Russia-Aligned Influence Operation Targets Germany </t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Sentinel Labs</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Commercial Threat Intel</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>45344</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>45231</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>45323</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>sources/SNT24.pdf</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sentinelone.com/labs/doppelganger-russia-aligned-influence-operation-targets-germany/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>REC23</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Obfuscation and AI Content in the Russian Influence Network ‚ÄúDoppelg√§nger‚Äù Signals Evolving Tactics</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Recorded Future</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Commercial Threat Intel</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>45265</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>45231</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>45231</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>sources/REC23.pdf</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.recordedfuture.com/research/russian-influence-network-doppelgangers-ai-content-tactics</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>SKY24</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Doppelg√§nger NG | Russian Cyberwarfare campaign</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>ClearSky Cyber Security</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Commercial Threat Intel</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>45344</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>45292</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>45323</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC; FR ABC</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>sources/SKY24.pdf</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.clearskysec.com/dg/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>ISD25</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Coordinated disinformation network uses AI, media impersonation to target German election</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Institute for Strategic Dialogue</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>NGO / Research</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>45701</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>45597</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>45687</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>DE AB</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>sources/ISD25.pdf</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.isdglobal.org/digital-dispatch/coordinated-disinformation-network-uses-ai-media-impersonation-to-target-german-election/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>REC25</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Stimmen aus Moskau: Russian Influence Operations Target German Elections</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Recorded Future</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Commercial Threat Intel</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>45701</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>45566</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>45689</v>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>sources/REC25.pdf</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.recordedfuture.com/research/stimmen-aus-moskau-russian-influence-operations-target-german-elections</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>CMS24</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>To be continued: The pro-Kremlin disinformation campaign Doppelganger in Germany</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>CeMAS</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>NGO / Research</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>45615</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>45231</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>45566</v>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC; FR AC; IT AC; PL AC</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>sources/CMS24.pdf</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>https://cemas.io/en/publications/to-be-continued-doppelganger-germany</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>CMS25-ENG</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Russische Desinformation vor der Bundestagswahl: Doppelg√§nger-Kampagne macht Stimmung gegen Parteien</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>CeMAS</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>NGO / Research</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>45677</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>45643</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>45671</v>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>DE ABC</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>sources/CMS25-ENG.pdf</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>https://btw2025.cemas.io/artikel/update-doppelgaenger</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>CHK25</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Influence by Design: Doppelg√§nger Sanctions, Meta and the Social Design Agency</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>CheckFirst</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Commercial Threat Intel</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>45658</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>44682</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>45566</v>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>FR AC; DE AC; IT AC; PL AC</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>sources/CHK25.pdf</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>https://checkfirst.network/wp-content/uploads/2025/01/Influence_by_Design.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>MET25</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Adversarial Threat Report, Fourth Quarter</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Platform Disclosure</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>45689</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>45566</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>45627</v>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>FR A; DE A; PL A</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>sources/MET25.pdf</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>https://transparency.meta.com/sr/Q4-2024-Adversarial-threat-report/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>MET24-2</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Q2_2023_Doppelganger_Russia_based_CIB_network_updated.csv</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Platform Disclosure</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>45629</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>44713</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>45597</v>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>FR AB; DE AB; IT AB; LV AB; PL AB</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>sources/MET24-2.csv</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/facebook/threat-research/blob/main/indicators/csv/Q2_2023%20/Q2_2023_Doppelganger_Russia_based_CIB_network_updated.csv</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>